<commit_message>
updated module to match with wtsp actual web propierties and created scripts for support mantainance
</commit_message>
<xml_diff>
--- a/contactos.xlsx
+++ b/contactos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Scripts_Python\VS_Code\Blitz_WASender\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://metso-my.sharepoint.com/personal/ricardo_uculmana_metso_com/Documents/Documents/VS Code/Blitz_WASender/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B0CEC4-1781-40F8-BD08-99F7B36B16EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{61040DA1-B0E5-4B12-B566-D98ECF03549B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B89E3B5-A84B-4E36-A16F-773DA871768E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C83D446C-466D-4BA9-B409-2D82AADD6820}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C83D446C-466D-4BA9-B409-2D82AADD6820}"/>
   </bookViews>
   <sheets>
     <sheet name="Contactos" sheetId="1" r:id="rId1"/>
@@ -30,9 +30,6 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -67,6 +64,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>{destinatario}</t>
@@ -88,6 +86,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> {remitente}</t>
@@ -108,6 +107,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>XXXX</t>
@@ -128,6 +128,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>XXXX</t>
@@ -150,6 +151,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>INSERTA AQUI TU ENLACE</t>
@@ -173,6 +175,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>{remitente}</t>
@@ -194,6 +197,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>XXXX</t>
@@ -215,6 +219,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>XXX</t>
@@ -230,6 +235,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>{destinatario}</t>
@@ -251,6 +257,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>XXXX</t>
@@ -273,6 +280,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>INSERTA AQUÍ TU ENLACE</t>
@@ -295,7 +303,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -308,6 +316,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -700,16 +709,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6849194-8580-456B-B6C5-EC63868F70E2}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="13.59765625" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.59765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.69921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -726,7 +735,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -743,7 +752,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -771,13 +780,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5822590-B957-46B2-9E7A-2E9D7A006E7A}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="71.5" customWidth="1"/>
+    <col min="1" max="1" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="71.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>4</v>
       </c>
@@ -785,7 +794,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="234.6">
+    <row r="2" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -793,7 +802,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="124.2">
+    <row r="3" spans="1:2" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>2</v>
       </c>

</xml_diff>